<commit_message>
Initial commit for Hackathon setup
</commit_message>
<xml_diff>
--- a/test-output/projectResourcesOutputs/GymsData.xlsx
+++ b/test-output/projectResourcesOutputs/GymsData.xlsx
@@ -41,22 +41,22 @@
     <t>08296044098</t>
   </si>
   <si>
-    <t>Vivek Teja's Human Weapon Fitness And Martial Arts</t>
+    <t>Berlin Fitness</t>
   </si>
   <si>
-    <t>09845459437</t>
-  </si>
-  <si>
-    <t>6E GYMS</t>
-  </si>
-  <si>
-    <t>07490833660</t>
+    <t>09008644895</t>
   </si>
   <si>
     <t>D'Shoolin Functional Strength &amp; therapy</t>
   </si>
   <si>
     <t>08401744248</t>
+  </si>
+  <si>
+    <t>Vivek Teja's Human Weapon Fitness And Martial Arts</t>
+  </si>
+  <si>
+    <t>09845459437</t>
   </si>
 </sst>
 </file>

</xml_diff>